<commit_message>
Avances con estadísticas y gráficas 2, Inferenciales
</commit_message>
<xml_diff>
--- a/RESULTADOS JUNIO/SEMAFORO LDA/TABLAS BONITAS JUN REV 1.xlsx
+++ b/RESULTADOS JUNIO/SEMAFORO LDA/TABLAS BONITAS JUN REV 1.xlsx
@@ -5,17 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\SEMAFORO LDA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\RESULTADOS JUNIO\SEMAFORO LDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E047C3A8-BF58-470A-B629-FE91F1E3B631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F34502-C376-43C1-9101-E062FE8DE812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="57600" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18750" yWindow="4770" windowWidth="57600" windowHeight="15345" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
+    <sheet name="Hoja5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="82">
   <si>
     <t>Case</t>
   </si>
@@ -144,13 +146,164 @@
   </si>
   <si>
     <t>X₂⁴</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Model Type</t>
+  </si>
+  <si>
+    <t>Non-linearty</t>
+  </si>
+  <si>
+    <t>Visualization (Projections)</t>
+  </si>
+  <si>
+    <t>LDA</t>
+  </si>
+  <si>
+    <t>Statistical</t>
+  </si>
+  <si>
+    <t>Linear</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>QDA</t>
+  </si>
+  <si>
+    <t>Quadratic</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>SVM (Poly 2)</t>
+  </si>
+  <si>
+    <t>Kernel-based</t>
+  </si>
+  <si>
+    <t>Hilbert Space (Degree 2)</t>
+  </si>
+  <si>
+    <t>SVM (Poly 3)</t>
+  </si>
+  <si>
+    <t>Hilbert Space (Degree 3)</t>
+  </si>
+  <si>
+    <t>SVM (RBF)</t>
+  </si>
+  <si>
+    <t>Hilbert Space (Radial Basis)</t>
+  </si>
+  <si>
+    <t>GNLPDA (Proposed)</t>
+  </si>
+  <si>
+    <t>stocastic</t>
+  </si>
+  <si>
+    <t>Non lineal</t>
+  </si>
+  <si>
+    <t>KFDA</t>
+  </si>
+  <si>
+    <t>Sí</t>
+  </si>
+  <si>
+    <t>LDA-M</t>
+  </si>
+  <si>
+    <t>GNLPDA (Propuesto)</t>
+  </si>
+  <si>
+    <t>Estocastico</t>
+  </si>
+  <si>
+    <t>No lineal</t>
+  </si>
+  <si>
+    <t>Espacio de Hilbert 
+(Radial Basis)</t>
+  </si>
+  <si>
+    <t>Espacio de Hilbert 
+(Grado 2)</t>
+  </si>
+  <si>
+    <t>Espacio de Hilbert 
+(Grado 3)</t>
+  </si>
+  <si>
+    <t>Método</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Tipo de modelo</t>
+  </si>
+  <si>
+    <t>No linealidad</t>
+  </si>
+  <si>
+    <t>Visualización</t>
+  </si>
+  <si>
+    <t>Estadístico</t>
+  </si>
+  <si>
+    <t>Basado en 
+Kernell</t>
+  </si>
+  <si>
+    <t>iris</t>
+  </si>
+  <si>
+    <t>penguins</t>
+  </si>
+  <si>
+    <t>pimadiabetes</t>
+  </si>
+  <si>
+    <t>wines</t>
+  </si>
+  <si>
+    <t>Cebolla3D</t>
+  </si>
+  <si>
+    <t>Cebolla10D</t>
+  </si>
+  <si>
+    <t>Cebolla20D</t>
+  </si>
+  <si>
+    <t>Breast Cancer (WDBC)</t>
+  </si>
+  <si>
+    <t>Ionosphere</t>
+  </si>
+  <si>
+    <t>Variables</t>
+  </si>
+  <si>
+    <t>Conjunto</t>
+  </si>
+  <si>
+    <t>Muestras</t>
+  </si>
+  <si>
+    <t>Clases</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,6 +350,28 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="17">
@@ -408,7 +583,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -425,30 +600,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -502,6 +653,51 @@
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -946,34 +1142,34 @@
       </c>
     </row>
     <row r="13" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="8"/>
-      <c r="M13" s="7" t="s">
+      <c r="L13" s="27"/>
+      <c r="M13" s="25" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="L14" s="9"/>
-      <c r="M14" s="6"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="26"/>
     </row>
     <row r="15" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="L15" s="10"/>
-      <c r="M15" s="7" t="s">
+      <c r="L15" s="29"/>
+      <c r="M15" s="25" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" spans="4:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L16" s="11"/>
-      <c r="M16" s="6"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="26"/>
     </row>
     <row r="17" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L17" s="12"/>
-      <c r="M17" s="7" t="s">
+      <c r="L17" s="31"/>
+      <c r="M17" s="25" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="18" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L18" s="13"/>
-      <c r="M18" s="6"/>
+      <c r="L18" s="32"/>
+      <c r="M18" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1140,22 +1336,22 @@
       </c>
     </row>
     <row r="12" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="N12" s="14"/>
+      <c r="N12" s="6"/>
     </row>
     <row r="13" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="N13" s="14"/>
+      <c r="N13" s="6"/>
     </row>
     <row r="14" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="N14" s="14"/>
+      <c r="N14" s="6"/>
     </row>
     <row r="15" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="M15" s="14"/>
+      <c r="M15" s="6"/>
     </row>
     <row r="16" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="M16" s="14"/>
+      <c r="M16" s="6"/>
     </row>
     <row r="17" spans="13:13" x14ac:dyDescent="0.25">
-      <c r="M17" s="14"/>
+      <c r="M17" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1169,165 +1365,551 @@
   <sheetData>
     <row r="3" spans="5:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="5:19" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="I4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="18" t="s">
+      <c r="K4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="18" t="s">
+      <c r="L4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="18" t="s">
+      <c r="M4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="18" t="s">
+      <c r="N4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="19" t="s">
+      <c r="O4" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="20" t="s">
+      <c r="P4" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="20" t="s">
+      <c r="Q4" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="R4" s="20" t="s">
+      <c r="R4" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="S4" s="20" t="s">
+      <c r="S4" s="12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" spans="5:19" ht="24.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E5" s="21">
+      <c r="E5" s="13">
         <v>1</v>
       </c>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="24"/>
-      <c r="P5" s="24"/>
-      <c r="Q5" s="24"/>
-      <c r="R5" s="24"/>
-      <c r="S5" s="24"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
+      <c r="S5" s="16"/>
     </row>
     <row r="6" spans="5:19" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E6" s="25">
+      <c r="E6" s="17">
         <v>2</v>
       </c>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="28"/>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="28"/>
-      <c r="R6" s="28"/>
-      <c r="S6" s="28"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
     </row>
     <row r="7" spans="5:19" ht="24.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E7" s="29">
+      <c r="E7" s="21">
         <v>3</v>
       </c>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="24"/>
-      <c r="P7" s="24"/>
-      <c r="Q7" s="24"/>
-      <c r="R7" s="24"/>
-      <c r="S7" s="24"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="16"/>
     </row>
     <row r="8" spans="5:19" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E8" s="25">
+      <c r="E8" s="17">
         <v>4</v>
       </c>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="27"/>
-      <c r="L8" s="27"/>
-      <c r="M8" s="27"/>
-      <c r="N8" s="27"/>
-      <c r="O8" s="28"/>
-      <c r="P8" s="28"/>
-      <c r="Q8" s="28"/>
-      <c r="R8" s="28"/>
-      <c r="S8" s="28"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+      <c r="S8" s="20"/>
     </row>
     <row r="9" spans="5:19" ht="24.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E9" s="29">
+      <c r="E9" s="21">
         <v>5</v>
       </c>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="24"/>
-      <c r="P9" s="24"/>
-      <c r="Q9" s="24"/>
-      <c r="R9" s="24"/>
-      <c r="S9" s="24"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+      <c r="S9" s="16"/>
     </row>
     <row r="10" spans="5:19" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E10" s="25">
+      <c r="E10" s="17">
         <v>6</v>
       </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="31"/>
-      <c r="M10" s="31"/>
-      <c r="N10" s="31"/>
-      <c r="O10" s="32"/>
-      <c r="P10" s="32"/>
-      <c r="Q10" s="32"/>
-      <c r="R10" s="32"/>
-      <c r="S10" s="32"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="24"/>
+      <c r="P10" s="24"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="24"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECA85A22-0E95-4C3C-B278-831FF15CAA60}">
+  <dimension ref="C3:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.140625" customWidth="1"/>
+    <col min="6" max="6" width="38.7109375" customWidth="1"/>
+    <col min="8" max="8" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="3:11" ht="53.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="J4" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="K4" s="33" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="3:11" ht="27.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="J5" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="J6" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" ht="80.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="K7" s="34" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="K8" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" ht="80.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="K9" s="34" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="I10" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="K10" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" ht="54" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="H11" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="I11" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="K11" s="34" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96D57A4-143A-46B9-B072-D3CCECD1B263}">
+  <dimension ref="C2:F12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="3:6" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="3:6" ht="27" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="38">
+        <v>150</v>
+      </c>
+      <c r="E4" s="38">
+        <v>4</v>
+      </c>
+      <c r="F4" s="38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="3:6" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="39">
+        <v>342</v>
+      </c>
+      <c r="E5" s="39">
+        <v>4</v>
+      </c>
+      <c r="F5" s="39">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" ht="27" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="38" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="38">
+        <v>768</v>
+      </c>
+      <c r="E6" s="38">
+        <v>8</v>
+      </c>
+      <c r="F6" s="38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="39" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="39">
+        <v>178</v>
+      </c>
+      <c r="E7" s="39">
+        <v>13</v>
+      </c>
+      <c r="F7" s="39">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" ht="27" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="38">
+        <v>300</v>
+      </c>
+      <c r="E8" s="38">
+        <v>3</v>
+      </c>
+      <c r="F8" s="38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="39">
+        <v>300</v>
+      </c>
+      <c r="E9" s="39">
+        <v>10</v>
+      </c>
+      <c r="F9" s="39">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" ht="27" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="38">
+        <v>300</v>
+      </c>
+      <c r="E10" s="38">
+        <v>20</v>
+      </c>
+      <c r="F10" s="38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="3:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="39" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="39">
+        <v>569</v>
+      </c>
+      <c r="E11" s="39">
+        <v>30</v>
+      </c>
+      <c r="F11" s="39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="3:6" ht="27" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="38">
+        <v>351</v>
+      </c>
+      <c r="E12" s="38">
+        <v>34</v>
+      </c>
+      <c r="F12" s="38">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>